<commit_message>
Corte del 1 de octubre: T02 recibida por correo
</commit_message>
<xml_diff>
--- a/calificaciones/P00-T02-corte-01oct.xlsx
+++ b/calificaciones/P00-T02-corte-01oct.xlsx
@@ -1099,7 +1099,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>NP</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Tu T01 ya está en Git, en tu carpeta: se queda en 8 por lo mismo que en el corte anterior (comentario de modelado, "// firma:" y un main por objeto). Falta la T02. La P04 vence el 9-oct.</t>
+          <t>T02 recibida por correo: el bisiesto da los cuatro casos bien y las letras salen correctas con if y con switch, salvo con 0, que responde "inválida" cuando el rango es de 0 a 100 y 0 es F; queda en 9. Súbela también a tu carpeta. Tu T01 ya está en Git y se queda en 8 (comentario de modelado, "// firma:" y un main por objeto). La P04 vence el 9-oct.</t>
         </is>
       </c>
     </row>

</xml_diff>